<commit_message>
ALL DOCS WORKING INITIAL
</commit_message>
<xml_diff>
--- a/input_data.xlsx
+++ b/input_data.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dharmesh\Desktop\Autofill\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A874BF-6F10-4611-88B8-2998629FFBD4}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57156785-4327-4F57-A540-C5EB152B9491}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" activeTab="1" xr2:uid="{4C90462E-EB49-4844-8D3D-C7A54EA72768}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" xr2:uid="{4C90462E-EB49-4844-8D3D-C7A54EA72768}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="3" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="41">
   <si>
     <t>SOLAR_CAPACITY</t>
   </si>
@@ -43,9 +43,6 @@
     <t>CONSUMER_APP_DATE</t>
   </si>
   <si>
-    <t>PANEL_CAPACITY</t>
-  </si>
-  <si>
     <t>PANEL_WATT</t>
   </si>
   <si>
@@ -58,18 +55,6 @@
     <t>CELL_MANUFACTURER</t>
   </si>
   <si>
-    <t>Indresh Devji Poladiya</t>
-  </si>
-  <si>
-    <t>Ganesh Cross Road Near Yogeshwar Medical Chalisgaon - 424101</t>
-  </si>
-  <si>
-    <t>Fujiyama Power System Private Limited</t>
-  </si>
-  <si>
-    <t>Mundra Solar Private Limited</t>
-  </si>
-  <si>
     <t>TOTAL_PANEL_CAPACITY</t>
   </si>
   <si>
@@ -77,16 +62,111 @@
   </si>
   <si>
     <t>123456, 123456, 123456, 123456, 123456, 123456</t>
+  </si>
+  <si>
+    <t>CONSUMER_NO</t>
+  </si>
+  <si>
+    <t>CONSUMER_PHONE</t>
+  </si>
+  <si>
+    <t>CONSUMER_EMAIL</t>
+  </si>
+  <si>
+    <t>SANCTIONED_CAPACITY</t>
+  </si>
+  <si>
+    <t>INSTALLATION_DATE</t>
+  </si>
+  <si>
+    <t>INVERTER_CAPACITY</t>
+  </si>
+  <si>
+    <t>INVERTER_MAKE</t>
+  </si>
+  <si>
+    <t>INSTALLATION_CITY</t>
+  </si>
+  <si>
+    <t>INSTALLATION_DISTRICT</t>
+  </si>
+  <si>
+    <t>CONSUMER_AADHAR</t>
+  </si>
+  <si>
+    <t>SANCTION_NUMBER</t>
+  </si>
+  <si>
+    <t>PANEL_GURANTEE</t>
+  </si>
+  <si>
+    <t>INVERTER_GURANTEE</t>
+  </si>
+  <si>
+    <t>Dharmesh Poladiya</t>
+  </si>
+  <si>
+    <t>Ganesh Cross road near yogeshwar medical</t>
+  </si>
+  <si>
+    <t>3150  Watt</t>
+  </si>
+  <si>
+    <t>UTL SOLAR</t>
+  </si>
+  <si>
+    <t>Mundra Solar PVT. LTD</t>
+  </si>
+  <si>
+    <t>dharmeshpoladiya75@gmail.com</t>
+  </si>
+  <si>
+    <t>UTL Solar</t>
+  </si>
+  <si>
+    <t>Chalisgaon</t>
+  </si>
+  <si>
+    <t>Jalgaon</t>
+  </si>
+  <si>
+    <t>1234-1234-1234</t>
+  </si>
+  <si>
+    <t>25 Years</t>
+  </si>
+  <si>
+    <t>21 Years</t>
+  </si>
+  <si>
+    <t>DISCOM_REGISTERED_OFFICE</t>
+  </si>
+  <si>
+    <t>Chalisgaon-U</t>
+  </si>
+  <si>
+    <t>Yug Poladiya</t>
+  </si>
+  <si>
+    <t>Indresh Poladiya</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -109,19 +189,25 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -433,146 +519,548 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EFEA3EC-3C76-41FC-B541-D604EB634AF0}">
-  <dimension ref="A1:A10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B87AFEC-6B2A-4D36-9588-F559C9B7DC78}">
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20" style="2" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="20.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="27.42578125" style="4" customWidth="1"/>
+    <col min="26" max="16384" width="9.140625" style="2"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y1" s="4" t="s">
+        <v>37</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1</v>
+    <row r="2" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="2">
+        <v>12345678</v>
+      </c>
+      <c r="E2" s="1">
+        <v>45658</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="2">
+        <v>6</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" s="2">
+        <v>525</v>
+      </c>
+      <c r="L2" s="2">
+        <v>12345678</v>
+      </c>
+      <c r="M2" s="2">
+        <v>7588647905</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="O2" s="2">
+        <v>3</v>
+      </c>
+      <c r="P2" s="1">
+        <v>45658</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>5</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="V2" s="2">
+        <v>123456778</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y2" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>2</v>
+    <row r="3" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A3" s="2">
+        <v>3</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="2">
+        <v>12345678</v>
+      </c>
+      <c r="E3" s="1">
+        <v>45658</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="2">
+        <v>6</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K3" s="2">
+        <v>525</v>
+      </c>
+      <c r="L3" s="2">
+        <v>12345678</v>
+      </c>
+      <c r="M3" s="2">
+        <v>7588647905</v>
+      </c>
+      <c r="N3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="O3" s="2">
+        <v>3</v>
+      </c>
+      <c r="P3" s="1">
+        <v>45658</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>5</v>
+      </c>
+      <c r="R3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="S3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="T3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="V3" s="2">
+        <v>123456778</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y3" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+    <row r="4" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="B4" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="2">
+        <v>12345678</v>
+      </c>
+      <c r="E4" s="1">
+        <v>45658</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="2">
+        <v>6</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K4" s="2">
+        <v>525</v>
+      </c>
+      <c r="L4" s="2">
+        <v>12345678</v>
+      </c>
+      <c r="M4" s="2">
+        <v>7588647905</v>
+      </c>
+      <c r="N4" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="O4" s="2">
+        <v>3</v>
+      </c>
+      <c r="P4" s="1">
+        <v>45658</v>
+      </c>
+      <c r="Q4" s="2">
         <v>5</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>9</v>
+      <c r="R4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="S4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="T4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="V4" s="2">
+        <v>123456778</v>
+      </c>
+      <c r="W4" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="X4" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y4" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="N2" r:id="rId1" xr:uid="{16ED03B9-0E3C-4A56-9425-80B55087A3B9}"/>
+    <hyperlink ref="N3" r:id="rId2" xr:uid="{35B17717-C809-4E37-810F-880561CA2DB5}"/>
+    <hyperlink ref="N4" r:id="rId3" xr:uid="{DBA254E0-2535-4EF8-8D94-E8290541558A}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F408F287-A46D-4D5C-97BD-AA37988BBF9F}">
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:Y2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="11" width="24.7109375" style="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="1"/>
+    <col min="1" max="1" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="21.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="14.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="17" style="2" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="20.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="18.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="22.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="19.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="22.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20" style="2" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="19.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="20.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="9.140625" style="4"/>
+    <col min="26" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="J1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="M1" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G1" s="1" t="s">
+      <c r="P1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="V1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="W1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="X1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y1" s="4" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:25" ht="90" x14ac:dyDescent="0.25">
+      <c r="A2" s="2">
+        <v>3</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D2" s="2">
+        <v>12345678</v>
+      </c>
+      <c r="E2" s="1">
+        <v>45658</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="2">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" ht="45" x14ac:dyDescent="0.25">
-      <c r="A2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="H2" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C2" s="1">
+      <c r="I2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="K2" s="2">
+        <v>525</v>
+      </c>
+      <c r="L2" s="2">
         <v>12345678</v>
       </c>
-      <c r="D2" s="2">
-        <v>45648</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" s="1">
-        <v>6</v>
-      </c>
-      <c r="G2" s="1">
-        <v>525</v>
-      </c>
-      <c r="H2" s="1">
-        <v>3150</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K2" s="1">
+      <c r="M2" s="2">
+        <v>7588647905</v>
+      </c>
+      <c r="N2" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="O2" s="2">
         <v>3</v>
+      </c>
+      <c r="P2" s="1">
+        <v>45658</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>5</v>
+      </c>
+      <c r="R2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="S2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="T2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="V2" s="2">
+        <v>123456778</v>
+      </c>
+      <c r="W2" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="Y2" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="N2" r:id="rId1" xr:uid="{B9947B28-0AEB-4299-960D-DF4223EB7634}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Added Meter Testing Document and updated other docs
</commit_message>
<xml_diff>
--- a/input_data.xlsx
+++ b/input_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dharmesh\Desktop\Autofill\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF66685-2620-4B44-87AC-E1CEDD27F32D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{218ED326-C1B9-42E6-A1EC-709A3EBD7606}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7545" xr2:uid="{4C90462E-EB49-4844-8D3D-C7A54EA72768}"/>
   </bookViews>
@@ -51,9 +51,6 @@
     <t>PANEL_COMPANY</t>
   </si>
   <si>
-    <t>CELL_MANUFACTURER</t>
-  </si>
-  <si>
     <t>TOTAL_PANEL_CAPACITY</t>
   </si>
   <si>
@@ -90,18 +87,12 @@
     <t>CONSUMER_AADHAR</t>
   </si>
   <si>
-    <t>SANCTION_NUMBER</t>
-  </si>
-  <si>
     <t>PANEL_GURANTEE</t>
   </si>
   <si>
     <t>INVERTER_GURANTEE</t>
   </si>
   <si>
-    <t>Mundra Solar PVT. LTD</t>
-  </si>
-  <si>
     <t>Chalisgaon</t>
   </si>
   <si>
@@ -120,9 +111,6 @@
     <t>10 Years</t>
   </si>
   <si>
-    <t>3150 Watt</t>
-  </si>
-  <si>
     <t>27 Years</t>
   </si>
   <si>
@@ -138,21 +126,12 @@
     <t>FXUS1332511B848</t>
   </si>
   <si>
-    <t>INVERTER_MPPT</t>
-  </si>
-  <si>
-    <t>70-500</t>
-  </si>
-  <si>
     <t>UTL</t>
   </si>
   <si>
     <t>SYSTEM_COST</t>
   </si>
   <si>
-    <t>Fujiyama Power Systems PVT. LTD.</t>
-  </si>
-  <si>
     <t>Shri Sanjay Kumar Jijabrao Deshmukh</t>
   </si>
   <si>
@@ -169,13 +148,34 @@
   </si>
   <si>
     <t>Gajanan Construction Chalisgaon - 424101</t>
+  </si>
+  <si>
+    <t>FX2S5324J1A1298</t>
+  </si>
+  <si>
+    <t>METER_TESTING_DATE</t>
+  </si>
+  <si>
+    <t>METER_RECIPT_NO</t>
+  </si>
+  <si>
+    <t>L&amp;T</t>
+  </si>
+  <si>
+    <t>A9094612</t>
+  </si>
+  <si>
+    <t>GENERATION_METER_MAKE</t>
+  </si>
+  <si>
+    <t>GENERATION_METER_NO</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -190,6 +190,18 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -213,7 +225,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -227,6 +239,8 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -542,7 +556,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B87AFEC-6B2A-4D36-9588-F559C9B7DC78}">
-  <dimension ref="A1:AB3"/>
+  <dimension ref="A1:AC3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.85546875" style="2" bestFit="1" customWidth="1"/>
@@ -554,29 +568,30 @@
     <col min="7" max="7" width="22.5703125" style="2" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="21.7109375" style="2" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="19.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.42578125" style="2" customWidth="1"/>
-    <col min="15" max="15" width="20.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.28515625" style="2" customWidth="1"/>
-    <col min="17" max="17" width="17" style="2" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="14.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="20.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="19.5703125" style="2" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="18.7109375" style="2" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="22.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="27.42578125" style="2" customWidth="1"/>
-    <col min="28" max="28" width="14.140625" style="2" customWidth="1"/>
-    <col min="29" max="16384" width="9.140625" style="2"/>
+    <col min="10" max="10" width="16.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20.28515625" style="2" customWidth="1"/>
+    <col min="15" max="15" width="17" style="2" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="12.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.140625" style="2" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="23.28515625" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="13.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="17.42578125" style="2" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="19.5703125" style="2" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="18.7109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.85546875" style="2" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="27.42578125" style="2" customWidth="1"/>
+    <col min="25" max="25" width="14.140625" style="2" customWidth="1"/>
+    <col min="26" max="26" width="21.85546875" style="2" customWidth="1"/>
+    <col min="27" max="27" width="18.42578125" style="2" customWidth="1"/>
+    <col min="28" max="28" width="26.5703125" style="2" customWidth="1"/>
+    <col min="29" max="29" width="24.140625" style="2" customWidth="1"/>
+    <col min="30" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:29" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>1</v>
       </c>
@@ -584,19 +599,19 @@
         <v>2</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>13</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>14</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>4</v>
@@ -605,75 +620,78 @@
         <v>3</v>
       </c>
       <c r="J1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="K1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="M1" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="K1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="L1" s="2" t="s">
+      <c r="N1" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="T1" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="U1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="V1" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="U1" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="V1" s="2" t="s">
-        <v>8</v>
-      </c>
       <c r="W1" s="2" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="X1" s="2" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="Y1" s="2" t="s">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="Z1" s="2" t="s">
-        <v>19</v>
+        <v>42</v>
       </c>
       <c r="AA1" s="2" t="s">
-        <v>27</v>
+        <v>43</v>
       </c>
       <c r="AB1" s="2" t="s">
-        <v>40</v>
+        <v>46</v>
+      </c>
+      <c r="AC1" s="2" t="s">
+        <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:28" ht="180" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:29" ht="180" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="C2" s="2">
         <v>9766801602</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="E2" s="4">
         <v>229009589042</v>
@@ -691,75 +709,79 @@
         <v>63098391</v>
       </c>
       <c r="J2" s="2">
-        <v>63098391</v>
-      </c>
-      <c r="K2" s="2">
         <v>3</v>
       </c>
-      <c r="L2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="M2" s="2">
+      <c r="K2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L2" s="2">
         <v>3.3</v>
       </c>
+      <c r="M2" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="N2" s="2" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="O2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P2" s="2">
+        <v>525</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>6</v>
+      </c>
+      <c r="R2" s="2" t="str">
+        <f>(P2*Q2)&amp;" WATT"</f>
+        <v>3150 WATT</v>
+      </c>
+      <c r="S2" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="P2" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="Q2" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="R2" s="2">
-        <v>525</v>
-      </c>
-      <c r="S2" s="2">
-        <v>6</v>
-      </c>
       <c r="T2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="U2" s="2" t="s">
-        <v>34</v>
+        <v>28</v>
+      </c>
+      <c r="U2" s="1">
+        <v>45753</v>
       </c>
       <c r="V2" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="W2" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="X2" s="1">
-        <v>45753</v>
-      </c>
-      <c r="Y2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="Z2" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="AA2" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB2" s="2">
+        <v>23</v>
+      </c>
+      <c r="X2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="Y2" s="2">
         <v>195000</v>
       </c>
+      <c r="Z2" s="1">
+        <v>45773</v>
+      </c>
+      <c r="AA2" s="5">
+        <v>1020477</v>
+      </c>
+      <c r="AB2" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC2" s="6" t="s">
+        <v>45</v>
+      </c>
     </row>
-    <row r="3" spans="1:28" ht="180" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:29" ht="180" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C3" s="2">
         <v>9860146641</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="E3" s="4">
         <v>783770372784</v>
@@ -777,58 +799,65 @@
         <v>62438999</v>
       </c>
       <c r="J3" s="2">
-        <v>62438999</v>
-      </c>
-      <c r="K3" s="2">
         <v>3</v>
       </c>
-      <c r="L3" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" s="2">
+      <c r="K3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="L3" s="2">
         <v>5.3</v>
       </c>
+      <c r="M3" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="N3" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P3" s="2">
+        <v>525</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>6</v>
+      </c>
+      <c r="R3" s="2" t="str">
+        <f>(P3*Q3)&amp;" WATT"</f>
+        <v>3150 WATT</v>
+      </c>
+      <c r="S3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="O3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="Q3" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="R3" s="2">
-        <v>525</v>
-      </c>
-      <c r="S3" s="2">
-        <v>6</v>
-      </c>
       <c r="T3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="U3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="U3" s="1">
+        <v>45741</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="W3" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="X3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="Y3" s="2">
+        <v>210000</v>
+      </c>
+      <c r="Z3" s="1">
+        <v>45773</v>
+      </c>
+      <c r="AA3" s="5">
+        <v>1020477</v>
+      </c>
+      <c r="AB3" s="5" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC3" s="6" t="s">
         <v>45</v>
-      </c>
-      <c r="V3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="W3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="X3" s="1">
-        <v>45741</v>
-      </c>
-      <c r="Y3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="Z3" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="AA3" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="AB3" s="2">
-        <v>210000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>